<commit_message>
Reorder monthly claim sheets: empty Latest Date Worked first, Finalized/PAID last
In every specialty sheet of the six monthly workbooks, rows with an empty
Latest Date Worked move to the top and Finalized and PAID claims move to
the bottom. The existing deadline order is kept within each group. The
Read Me row-order section is updated to match. The master is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 02 February.xlsx
+++ b/SPC26S1 - 02 February.xlsx
@@ -1844,13 +1844,13 @@
     <t>39 claims with a date of service in 2026-02 February, split into one sheet per specialty: BH, DME, GAE, ORTHO, US.</t>
   </si>
   <si>
-    <t>Row order - timely filing deadline</t>
-  </si>
-  <si>
-    <t>Every specialty sheet is sorted by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: claims with five days or less left sit at the top of each sheet in red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
-  </si>
-  <si>
-    <t>Order down the sheet, with the colour band each row gets, counted on 19 September 2026:</t>
+    <t>Row order - work queue, then timely filing deadline</t>
+  </si>
+  <si>
+    <t>Every specialty sheet is sorted in three groups: claims with an empty Latest Date Worked (column K) at the top, then the other open claims, and Finalized and PAID claims at the bottom (a Finalized or PAID claim goes to the bottom even when its Latest Date Worked is empty). Within each group, rows are ordered by how close the claim is to its primary payer's timely filing deadline. Days Until Deadline (column L) carries the count: five days or less left is shaded red, a negative number means the filing window has already closed, and a blank means no limit is on file for that payer.</t>
+  </si>
+  <si>
+    <t>Deadline order within each group, with the colour band each row gets, counted on 19 September 2026:</t>
   </si>
   <si>
     <t xml:space="preserve">    1 - Due in 5 days or less: 0</t>
@@ -1871,7 +1871,7 @@
     <t>Past due rows sit below the claims that can still be filed on time rather than at the very top, so the actionable work stays first. That is why the numbers run up to the longest window and then restart at the negatives.</t>
   </si>
   <si>
-    <t>Filing Deadline is the date of service plus the primary payer's limit, taken from 'Carrier_Timely_Filing_Reference.xlsx'. Days Until Deadline is a live formula, so the count stays true as time passes - but the row order is a snapshot taken on 12 August 2026. Sort ascending on Days Until Deadline to bring the order up to date; that puts the past due rows first.</t>
+    <t>Filing Deadline is the date of service plus the primary payer's limit, taken from 'Carrier_Timely_Filing_Reference.xlsx'. Days Until Deadline is a live formula, so the count stays true as time passes - but the row order is a snapshot taken on 12 August 2026. Sorting on Days Until Deadline alone would mix the three groups above back together, so when you re-sort keep the empty Latest Date Worked rows first and the Finalized and PAID rows last.</t>
   </si>
   <si>
     <t>Where a payer had two possible limits the shorter one was used, so the real deadline can only be later, never earlier. Filing Limit and Limit Carrier name the figure applied and the carrier row it came from.</t>
@@ -3661,7 +3661,7 @@
         <v>46183</v>
       </c>
       <c r="L2" s="12">
-        <f t="shared" ref="L2:L9" ca="1" si="0">IF($O2="","",$O2-TODAY())</f>
+        <f ca="1">IF($O2="","",$O2-TODAY())</f>
         <v>-154</v>
       </c>
       <c r="M2" s="12">
@@ -3669,7 +3669,7 @@
         <v>-154</v>
       </c>
       <c r="N2" s="12">
-        <f t="shared" ref="N2:N9" ca="1" si="1">IF($C2="","",$C2+365-TODAY())</f>
+        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
         <v>163</v>
       </c>
       <c r="O2" s="6">
@@ -3772,7 +3772,7 @@
         <v>46183</v>
       </c>
       <c r="L3" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O3="","",$O3-TODAY())</f>
         <v>-148</v>
       </c>
       <c r="M3" s="12">
@@ -3780,7 +3780,7 @@
         <v>-148</v>
       </c>
       <c r="N3" s="12">
-        <f t="shared" ca="1" si="1"/>
+        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
         <v>213</v>
       </c>
       <c r="O3" s="6">
@@ -3850,60 +3850,64 @@
     </row>
     <row r="4" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="C4" s="3">
-        <v>46119</v>
+        <v>46147</v>
       </c>
       <c r="D4" s="4">
-        <v>549765437</v>
+        <v>557794433</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F4" s="6">
-        <v>46065</v>
+        <v>46066</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="K4" s="3"/>
+        <v>69</v>
+      </c>
+      <c r="K4" s="3">
+        <v>46142</v>
+      </c>
       <c r="L4" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-145</v>
+        <f ca="1">IF($O4="","",$O4-TODAY())</f>
+        <v>-144</v>
       </c>
       <c r="M4" s="12">
-        <f ca="1">IF($F4="","",$F4+90-TODAY())</f>
-        <v>-145</v>
+        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <v>212</v>
       </c>
       <c r="N4" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>184</v>
+        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
+        <v>212</v>
       </c>
       <c r="O4" s="6">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="P4" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="T4" s="5" t="s">
         <v>49</v>
@@ -3918,37 +3922,35 @@
         <v>51</v>
       </c>
       <c r="Z4" s="7">
-        <v>1372.91</v>
+        <v>976.64</v>
       </c>
       <c r="AA4" s="7">
-        <v>1179.8900000000001</v>
+        <v>0</v>
       </c>
       <c r="AB4" s="7">
         <v>0</v>
       </c>
       <c r="AC4" s="6">
-        <v>46119</v>
+        <v>46147</v>
       </c>
       <c r="AD4" s="7">
-        <v>193.02</v>
+        <v>976.64</v>
       </c>
       <c r="AE4" s="4">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="AG4" s="5"/>
       <c r="AH4" s="5"/>
       <c r="AI4" s="5"/>
-      <c r="AJ4" s="4">
-        <v>558453526</v>
-      </c>
+      <c r="AJ4" s="4"/>
       <c r="AK4" s="5" t="s">
         <v>53</v>
       </c>
       <c r="AL4" s="5" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="AM4" s="6">
         <v>46086</v>
@@ -3961,20 +3963,20 @@
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>66</v>
+      <c r="B5" s="13" t="s">
+        <v>305</v>
       </c>
       <c r="C5" s="3">
         <v>46147</v>
       </c>
       <c r="D5" s="4">
-        <v>557794433</v>
+        <v>557794882</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F5" s="6">
-        <v>46066</v>
+        <v>46070</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>68</v>
@@ -3989,22 +3991,22 @@
         <v>69</v>
       </c>
       <c r="K5" s="3">
-        <v>46142</v>
+        <v>46284</v>
       </c>
       <c r="L5" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-144</v>
+        <f ca="1">IF($O5="","",$O5-TODAY())</f>
+        <v>-140</v>
       </c>
       <c r="M5" s="12">
         <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
         <v>212</v>
       </c>
       <c r="N5" s="12">
-        <f t="shared" ca="1" si="1"/>
+        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
         <v>212</v>
       </c>
       <c r="O5" s="6">
-        <v>46156</v>
+        <v>46160</v>
       </c>
       <c r="P5" s="5" t="s">
         <v>46</v>
@@ -4046,20 +4048,22 @@
         <v>976.64</v>
       </c>
       <c r="AE5" s="4">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AF5" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="AG5" s="5"/>
+        <v>74</v>
+      </c>
+      <c r="AG5" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
       <c r="AJ5" s="4"/>
       <c r="AK5" s="5" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="AL5" s="5" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="AM5" s="6">
         <v>46086</v>
@@ -4072,62 +4076,62 @@
       <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>305</v>
+      <c r="B6" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="C6" s="3">
-        <v>46147</v>
+        <v>46101</v>
       </c>
       <c r="D6" s="4">
-        <v>557794882</v>
+        <v>550288006</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F6" s="6">
-        <v>46070</v>
+        <v>46071</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="K6" s="3">
-        <v>46284</v>
+        <v>46183</v>
       </c>
       <c r="L6" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-140</v>
+        <f ca="1">IF($O6="","",$O6-TODAY())</f>
+        <v>-139</v>
       </c>
       <c r="M6" s="12">
+        <f ca="1">IF($F6="","",$F6+90-TODAY())</f>
+        <v>-139</v>
+      </c>
+      <c r="N6" s="12">
         <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>212</v>
-      </c>
-      <c r="N6" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>212</v>
+        <v>166</v>
       </c>
       <c r="O6" s="6">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="P6" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>49</v>
@@ -4139,10 +4143,10 @@
       <c r="W6" s="5"/>
       <c r="X6" s="5"/>
       <c r="Y6" s="5" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="Z6" s="7">
-        <v>976.64</v>
+        <v>1822.52</v>
       </c>
       <c r="AA6" s="7">
         <v>0</v>
@@ -4151,28 +4155,26 @@
         <v>0</v>
       </c>
       <c r="AC6" s="6">
-        <v>46147</v>
+        <v>46101</v>
       </c>
       <c r="AD6" s="7">
-        <v>976.64</v>
+        <v>1822.52</v>
       </c>
       <c r="AE6" s="4">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="AG6" s="5" t="s">
-        <v>64</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="AG6" s="5"/>
       <c r="AH6" s="5"/>
       <c r="AI6" s="5"/>
       <c r="AJ6" s="4"/>
       <c r="AK6" s="5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="AM6" s="6">
         <v>46086</v>
@@ -4186,61 +4188,61 @@
         <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C7" s="3">
-        <v>46101</v>
+        <v>46147</v>
       </c>
       <c r="D7" s="4">
-        <v>550288006</v>
+        <v>557793858</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F7" s="6">
-        <v>46071</v>
+        <v>46073</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="K7" s="3">
-        <v>46183</v>
+        <v>46266</v>
       </c>
       <c r="L7" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-139</v>
+        <f ca="1">IF($O7="","",$O7-TODAY())</f>
+        <v>-137</v>
       </c>
       <c r="M7" s="12">
-        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
-        <v>-139</v>
+        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <v>212</v>
       </c>
       <c r="N7" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>166</v>
+        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
+        <v>212</v>
       </c>
       <c r="O7" s="6">
-        <v>46161</v>
+        <v>46163</v>
       </c>
       <c r="P7" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="T7" s="5" t="s">
         <v>49</v>
@@ -4252,10 +4254,10 @@
       <c r="W7" s="5"/>
       <c r="X7" s="5"/>
       <c r="Y7" s="5" t="s">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="Z7" s="7">
-        <v>1822.52</v>
+        <v>976.64</v>
       </c>
       <c r="AA7" s="7">
         <v>0</v>
@@ -4264,26 +4266,26 @@
         <v>0</v>
       </c>
       <c r="AC7" s="6">
-        <v>46101</v>
+        <v>46147</v>
       </c>
       <c r="AD7" s="7">
-        <v>1822.52</v>
+        <v>976.64</v>
       </c>
       <c r="AE7" s="4">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="AF7" s="5" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="AG7" s="5"/>
       <c r="AH7" s="5"/>
       <c r="AI7" s="5"/>
       <c r="AJ7" s="4"/>
       <c r="AK7" s="5" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="AL7" s="5" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="AM7" s="6">
         <v>46086</v>
@@ -4297,16 +4299,16 @@
         <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" s="3">
         <v>46147</v>
       </c>
       <c r="D8" s="4">
-        <v>557793858</v>
+        <v>557794229</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F8" s="6">
         <v>46073</v>
@@ -4324,10 +4326,10 @@
         <v>69</v>
       </c>
       <c r="K8" s="3">
-        <v>46266</v>
+        <v>46247</v>
       </c>
       <c r="L8" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O8="","",$O8-TODAY())</f>
         <v>-137</v>
       </c>
       <c r="M8" s="12">
@@ -4335,7 +4337,7 @@
         <v>212</v>
       </c>
       <c r="N8" s="12">
-        <f t="shared" ca="1" si="1"/>
+        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
         <v>212</v>
       </c>
       <c r="O8" s="6">
@@ -4391,7 +4393,7 @@
       <c r="AI8" s="5"/>
       <c r="AJ8" s="4"/>
       <c r="AK8" s="5" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="AL8" s="5" t="s">
         <v>72</v>
@@ -4405,64 +4407,60 @@
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="B9" s="2"/>
       <c r="C9" s="3">
-        <v>46147</v>
+        <v>46119</v>
       </c>
       <c r="D9" s="4">
-        <v>557794229</v>
+        <v>549765437</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="F9" s="6">
-        <v>46073</v>
+        <v>46065</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="K9" s="3">
-        <v>46247</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="K9" s="3"/>
       <c r="L9" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-137</v>
+        <f ca="1">IF($O9="","",$O9-TODAY())</f>
+        <v>-145</v>
       </c>
       <c r="M9" s="12">
+        <f ca="1">IF($F9="","",$F9+90-TODAY())</f>
+        <v>-145</v>
+      </c>
+      <c r="N9" s="12">
         <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
-        <v>212</v>
-      </c>
-      <c r="N9" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>212</v>
+        <v>184</v>
       </c>
       <c r="O9" s="6">
-        <v>46163</v>
+        <v>46155</v>
       </c>
       <c r="P9" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="S9" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="T9" s="5" t="s">
         <v>49</v>
@@ -4477,35 +4475,37 @@
         <v>51</v>
       </c>
       <c r="Z9" s="7">
-        <v>976.64</v>
+        <v>1372.91</v>
       </c>
       <c r="AA9" s="7">
-        <v>0</v>
+        <v>1179.8900000000001</v>
       </c>
       <c r="AB9" s="7">
         <v>0</v>
       </c>
       <c r="AC9" s="6">
-        <v>46147</v>
+        <v>46119</v>
       </c>
       <c r="AD9" s="7">
-        <v>976.64</v>
+        <v>193.02</v>
       </c>
       <c r="AE9" s="4">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="AF9" s="5" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="AG9" s="5"/>
       <c r="AH9" s="5"/>
       <c r="AI9" s="5"/>
-      <c r="AJ9" s="4"/>
+      <c r="AJ9" s="4">
+        <v>558453526</v>
+      </c>
       <c r="AK9" s="5" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="AL9" s="5" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="AM9" s="6">
         <v>46086</v>
@@ -4786,52 +4786,50 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C2" s="3">
-        <v>46105</v>
+        <v>46147</v>
       </c>
       <c r="D2" s="4">
-        <v>553137846</v>
+        <v>557715576</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="F2" s="6">
-        <v>46063</v>
+        <v>46076</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>88</v>
+        <v>128</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="K2" s="3">
-        <v>46300</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="K2" s="3"/>
       <c r="L2" s="12">
-        <f t="shared" ref="L2:L12" ca="1" si="0">IF($O2="","",$O2-TODAY())</f>
-        <v>128</v>
+        <f ca="1">IF($O2="","",$O2-TODAY())</f>
+        <v>141</v>
       </c>
       <c r="M2" s="12">
-        <f t="shared" ref="M2:M8" ca="1" si="1">IF($C2="","",$C2+365-TODAY())</f>
-        <v>170</v>
+        <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
+        <v>212</v>
       </c>
       <c r="N2" s="12">
-        <f t="shared" ref="N2:N8" ca="1" si="2">IF($C2="","",$C2+120-TODAY())</f>
-        <v>-75</v>
+        <f ca="1">IF($C2="","",$C2+120-TODAY())</f>
+        <v>-33</v>
       </c>
       <c r="O2" s="6">
-        <v>46428</v>
+        <v>46441</v>
       </c>
       <c r="P2" s="5" t="s">
         <v>49</v>
@@ -4852,48 +4850,48 @@
         <v>50</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="Z2" s="7">
-        <v>5916.4</v>
+        <v>72707.600000000006</v>
       </c>
       <c r="AA2" s="7">
-        <v>5047.72</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="7">
-        <v>692.12</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="6">
-        <v>46105</v>
+        <v>46147</v>
       </c>
       <c r="AD2" s="7">
-        <v>176.56</v>
+        <v>72707.600000000006</v>
       </c>
       <c r="AE2" s="4">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="AF2" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="AG2" s="5"/>
+      <c r="AG2" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="AH2" s="5"/>
       <c r="AI2" s="5"/>
-      <c r="AJ2" s="4">
-        <v>564731184</v>
-      </c>
+      <c r="AJ2" s="4"/>
       <c r="AK2" s="5" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="AL2" s="5" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
       <c r="AM2" s="6">
-        <v>46099</v>
+        <v>46085</v>
       </c>
       <c r="AN2" s="5" t="s">
         <v>97</v>
@@ -4901,49 +4899,49 @@
     </row>
     <row r="3" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>203</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C3" s="3">
-        <v>46133</v>
+        <v>46105</v>
       </c>
       <c r="D3" s="4">
-        <v>553677900</v>
+        <v>553137846</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F3" s="6">
         <v>46063</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>88</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="K3" s="3">
         <v>46300</v>
       </c>
       <c r="L3" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O3="","",$O3-TODAY())</f>
         <v>128</v>
       </c>
       <c r="M3" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>198</v>
+        <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
+        <v>170</v>
       </c>
       <c r="N3" s="12">
-        <f t="shared" ca="1" si="2"/>
-        <v>-47</v>
+        <f ca="1">IF($C3="","",$C3+120-TODAY())</f>
+        <v>-75</v>
       </c>
       <c r="O3" s="6">
         <v>46428</v>
@@ -4967,7 +4965,7 @@
         <v>50</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
@@ -4978,16 +4976,16 @@
         <v>5916.4</v>
       </c>
       <c r="AA3" s="7">
-        <v>0</v>
+        <v>5047.72</v>
       </c>
       <c r="AB3" s="7">
-        <v>0</v>
+        <v>692.12</v>
       </c>
       <c r="AC3" s="6">
-        <v>46133</v>
+        <v>46105</v>
       </c>
       <c r="AD3" s="7">
-        <v>5916.4</v>
+        <v>176.56</v>
       </c>
       <c r="AE3" s="4">
         <v>179</v>
@@ -4998,7 +4996,9 @@
       <c r="AG3" s="5"/>
       <c r="AH3" s="5"/>
       <c r="AI3" s="5"/>
-      <c r="AJ3" s="4"/>
+      <c r="AJ3" s="4">
+        <v>564731184</v>
+      </c>
       <c r="AK3" s="5" t="s">
         <v>95</v>
       </c>
@@ -5006,7 +5006,7 @@
         <v>96</v>
       </c>
       <c r="AM3" s="6">
-        <v>46105</v>
+        <v>46099</v>
       </c>
       <c r="AN3" s="5" t="s">
         <v>97</v>
@@ -5047,15 +5047,15 @@
         <v>46300</v>
       </c>
       <c r="L4" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O4="","",$O4-TODAY())</f>
         <v>131</v>
       </c>
       <c r="M4" s="12">
-        <f t="shared" ca="1" si="1"/>
+        <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
         <v>198</v>
       </c>
       <c r="N4" s="12">
-        <f t="shared" ca="1" si="2"/>
+        <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
         <v>-47</v>
       </c>
       <c r="O4" s="6">
@@ -5133,67 +5133,67 @@
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>61</v>
+        <v>131</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="C5" s="3">
-        <v>46133</v>
+        <v>46227</v>
       </c>
       <c r="D5" s="4">
-        <v>551104780</v>
+        <v>565140993</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="F5" s="6">
         <v>46069</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>107</v>
+        <v>44</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="K5" s="3">
-        <v>46261</v>
+        <v>46196</v>
       </c>
       <c r="L5" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>134</v>
+        <f ca="1">IF($O5="","",$O5-TODAY())</f>
+        <v>-141</v>
       </c>
       <c r="M5" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>198</v>
+        <f ca="1">IF($F5="","",$F5+90-TODAY())</f>
+        <v>-141</v>
       </c>
       <c r="N5" s="12">
-        <f t="shared" ca="1" si="2"/>
-        <v>-47</v>
+        <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
+        <v>292</v>
       </c>
       <c r="O5" s="6">
-        <v>46434</v>
+        <v>46159</v>
       </c>
       <c r="P5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="T5" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="U5" s="5" t="s">
         <v>50</v>
@@ -5201,49 +5201,41 @@
       <c r="V5" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="W5" s="5" t="s">
-        <v>110</v>
-      </c>
+      <c r="W5" s="5"/>
       <c r="X5" s="5"/>
       <c r="Y5" s="5" t="s">
         <v>51</v>
       </c>
       <c r="Z5" s="7">
-        <v>1082.98</v>
+        <v>5492.55</v>
       </c>
       <c r="AA5" s="7">
-        <v>17.32</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="7">
-        <v>849.06</v>
-      </c>
-      <c r="AC5" s="6">
-        <v>46133</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="6"/>
       <c r="AD5" s="7">
-        <v>216.6</v>
+        <v>5492.55</v>
       </c>
       <c r="AE5" s="4">
         <v>173</v>
       </c>
       <c r="AF5" s="5" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="AG5" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="AH5" s="5" t="s">
-        <v>113</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
-      <c r="AJ5" s="4">
-        <v>566111704</v>
-      </c>
+      <c r="AJ5" s="4"/>
       <c r="AK5" s="5" t="s">
-        <v>95</v>
+        <v>137</v>
       </c>
       <c r="AL5" s="5" t="s">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="AM5" s="6">
         <v>46080</v>
@@ -5254,116 +5246,114 @@
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>310</v>
+        <v>139</v>
       </c>
       <c r="C6" s="3">
-        <v>46121</v>
+        <v>46106</v>
       </c>
       <c r="D6" s="4">
-        <v>553095408</v>
+        <v>550530483</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="F6" s="6">
-        <v>46069</v>
+        <v>46072</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>88</v>
+        <v>141</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>116</v>
+        <v>44</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="K6" s="3">
-        <v>46246</v>
+        <v>46197</v>
       </c>
       <c r="L6" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>134</v>
+        <f ca="1">IF($O6="","",$O6-TODAY())</f>
+        <v>-138</v>
       </c>
       <c r="M6" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>186</v>
+        <f ca="1">IF($C6="","",$C6+180-TODAY())</f>
+        <v>-14</v>
       </c>
       <c r="N6" s="12">
-        <f t="shared" ca="1" si="2"/>
-        <v>-59</v>
+        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <v>171</v>
       </c>
       <c r="O6" s="6">
-        <v>46434</v>
+        <v>46162</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="S6" s="5" t="s">
         <v>50</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>50</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="W6" s="5"/>
       <c r="X6" s="5"/>
       <c r="Y6" s="5" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="Z6" s="7">
-        <v>18176.900000000001</v>
+        <v>5916.4</v>
       </c>
       <c r="AA6" s="7">
-        <v>15508.1</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="7">
-        <v>542.44000000000005</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="6">
-        <v>46121</v>
+        <v>46106</v>
       </c>
       <c r="AD6" s="7">
-        <v>2126.36</v>
+        <v>5916.4</v>
       </c>
       <c r="AE6" s="4">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="AF6" s="5" t="s">
         <v>94</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="AH6" s="5"/>
       <c r="AI6" s="5"/>
-      <c r="AJ6" s="4">
-        <v>557144068</v>
-      </c>
+      <c r="AJ6" s="4"/>
       <c r="AK6" s="5" t="s">
-        <v>119</v>
+        <v>145</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="AM6" s="6">
-        <v>46099</v>
+        <v>46077</v>
       </c>
       <c r="AN6" s="5" t="s">
         <v>97</v>
@@ -5371,81 +5361,63 @@
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>311</v>
+        <v>146</v>
       </c>
       <c r="C7" s="3">
-        <v>46101</v>
+        <v>46149</v>
       </c>
       <c r="D7" s="4">
-        <v>550127169</v>
+        <v>556897081</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
       <c r="F7" s="6">
-        <v>46071</v>
+        <v>46062</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>88</v>
+        <v>148</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>88</v>
+        <v>148</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>122</v>
+        <v>44</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="K7" s="3">
-        <v>46300</v>
-      </c>
-      <c r="L7" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>136</v>
-      </c>
-      <c r="M7" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>166</v>
-      </c>
-      <c r="N7" s="12">
-        <f t="shared" ca="1" si="2"/>
-        <v>-79</v>
-      </c>
-      <c r="O7" s="6">
-        <v>46436</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>49</v>
-      </c>
+        <v>46134</v>
+      </c>
+      <c r="L7" s="12" t="str">
+        <f ca="1">IF($O7="","",$O7-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="5"/>
       <c r="Q7" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="T7" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="U7" s="5" t="s">
-        <v>50</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
       <c r="V7" s="5" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="W7" s="5"/>
       <c r="X7" s="5"/>
       <c r="Y7" s="5" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="Z7" s="7">
-        <v>6392.96</v>
+        <v>5424.4</v>
       </c>
       <c r="AA7" s="7">
         <v>0</v>
@@ -5454,29 +5426,29 @@
         <v>0</v>
       </c>
       <c r="AC7" s="6">
-        <v>46101</v>
+        <v>46149</v>
       </c>
       <c r="AD7" s="7">
-        <v>6392.96</v>
+        <v>5424.4</v>
       </c>
       <c r="AE7" s="4">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="AF7" s="5" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="AG7" s="5"/>
       <c r="AH7" s="5"/>
       <c r="AI7" s="5"/>
       <c r="AJ7" s="4"/>
       <c r="AK7" s="5" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="AL7" s="5" t="s">
-        <v>126</v>
+        <v>54</v>
       </c>
       <c r="AM7" s="6">
-        <v>46093</v>
+        <v>46063</v>
       </c>
       <c r="AN7" s="5" t="s">
         <v>97</v>
@@ -5487,76 +5459,60 @@
         <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>312</v>
+        <v>152</v>
       </c>
       <c r="C8" s="3">
-        <v>46147</v>
+        <v>46112</v>
       </c>
       <c r="D8" s="4">
-        <v>557715576</v>
+        <v>553079628</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="F8" s="6">
-        <v>46076</v>
+        <v>46064</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="K8" s="3"/>
-      <c r="L8" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>141</v>
-      </c>
-      <c r="M8" s="12">
-        <f t="shared" ca="1" si="1"/>
-        <v>212</v>
-      </c>
-      <c r="N8" s="12">
-        <f t="shared" ca="1" si="2"/>
-        <v>-33</v>
-      </c>
-      <c r="O8" s="6">
-        <v>46441</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>49</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="K8" s="3">
+        <v>46244</v>
+      </c>
+      <c r="L8" s="12" t="str">
+        <f ca="1">IF($O8="","",$O8-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="5"/>
       <c r="Q8" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="T8" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="U8" s="5" t="s">
-        <v>50</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
       <c r="V8" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="W8" s="5"/>
       <c r="X8" s="5"/>
       <c r="Y8" s="5" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="Z8" s="7">
-        <v>72707.600000000006</v>
+        <v>18176.900000000001</v>
       </c>
       <c r="AA8" s="7">
         <v>0</v>
@@ -5565,31 +5521,31 @@
         <v>0</v>
       </c>
       <c r="AC8" s="6">
-        <v>46147</v>
+        <v>46112</v>
       </c>
       <c r="AD8" s="7">
-        <v>72707.600000000006</v>
+        <v>18176.900000000001</v>
       </c>
       <c r="AE8" s="4">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="AF8" s="5" t="s">
         <v>94</v>
       </c>
       <c r="AG8" s="5" t="s">
-        <v>105</v>
+        <v>155</v>
       </c>
       <c r="AH8" s="5"/>
       <c r="AI8" s="5"/>
       <c r="AJ8" s="4"/>
       <c r="AK8" s="5" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="AL8" s="5" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="AM8" s="6">
-        <v>46085</v>
+        <v>46099</v>
       </c>
       <c r="AN8" s="5" t="s">
         <v>97</v>
@@ -5597,81 +5553,81 @@
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>131</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>132</v>
+        <v>308</v>
       </c>
       <c r="C9" s="3">
-        <v>46227</v>
+        <v>46133</v>
       </c>
       <c r="D9" s="4">
-        <v>565140993</v>
+        <v>553677900</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>133</v>
+        <v>98</v>
       </c>
       <c r="F9" s="6">
-        <v>46069</v>
+        <v>46063</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="J9" s="5" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="K9" s="3">
-        <v>46196</v>
+        <v>46300</v>
       </c>
       <c r="L9" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-141</v>
+        <f ca="1">IF($O9="","",$O9-TODAY())</f>
+        <v>128</v>
       </c>
       <c r="M9" s="12">
-        <f ca="1">IF($F9="","",$F9+90-TODAY())</f>
-        <v>-141</v>
+        <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
+        <v>198</v>
       </c>
       <c r="N9" s="12">
-        <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
-        <v>292</v>
+        <f ca="1">IF($C9="","",$C9+120-TODAY())</f>
+        <v>-47</v>
       </c>
       <c r="O9" s="6">
-        <v>46159</v>
+        <v>46428</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="S9" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="U9" s="5" t="s">
         <v>50</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="W9" s="5"/>
       <c r="X9" s="5"/>
       <c r="Y9" s="5" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="Z9" s="7">
-        <v>5492.55</v>
+        <v>5916.4</v>
       </c>
       <c r="AA9" s="7">
         <v>0</v>
@@ -5679,30 +5635,30 @@
       <c r="AB9" s="7">
         <v>0</v>
       </c>
-      <c r="AC9" s="6"/>
+      <c r="AC9" s="6">
+        <v>46133</v>
+      </c>
       <c r="AD9" s="7">
-        <v>5492.55</v>
+        <v>5916.4</v>
       </c>
       <c r="AE9" s="4">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="AF9" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="AG9" s="5" t="s">
-        <v>136</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="AG9" s="5"/>
       <c r="AH9" s="5"/>
       <c r="AI9" s="5"/>
       <c r="AJ9" s="4"/>
       <c r="AK9" s="5" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="AL9" s="5" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="AM9" s="6">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="AN9" s="5" t="s">
         <v>97</v>
@@ -5710,114 +5666,120 @@
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="C10" s="3">
-        <v>46106</v>
+        <v>46133</v>
       </c>
       <c r="D10" s="4">
-        <v>550530483</v>
+        <v>551104780</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="F10" s="6">
-        <v>46072</v>
+        <v>46069</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>141</v>
+        <v>88</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="K10" s="3">
-        <v>46197</v>
+        <v>46261</v>
       </c>
       <c r="L10" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-138</v>
+        <f ca="1">IF($O10="","",$O10-TODAY())</f>
+        <v>134</v>
       </c>
       <c r="M10" s="12">
-        <f ca="1">IF($C10="","",$C10+180-TODAY())</f>
-        <v>-14</v>
+        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
+        <v>198</v>
       </c>
       <c r="N10" s="12">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>171</v>
+        <f ca="1">IF($C10="","",$C10+120-TODAY())</f>
+        <v>-47</v>
       </c>
       <c r="O10" s="6">
-        <v>46162</v>
+        <v>46434</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>142</v>
+        <v>90</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>143</v>
+        <v>49</v>
       </c>
       <c r="S10" s="5" t="s">
         <v>50</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="U10" s="5" t="s">
         <v>50</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="W10" s="5"/>
+        <v>109</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="X10" s="5"/>
       <c r="Y10" s="5" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="Z10" s="7">
-        <v>5916.4</v>
+        <v>1082.98</v>
       </c>
       <c r="AA10" s="7">
-        <v>0</v>
+        <v>17.32</v>
       </c>
       <c r="AB10" s="7">
-        <v>0</v>
+        <v>849.06</v>
       </c>
       <c r="AC10" s="6">
-        <v>46106</v>
+        <v>46133</v>
       </c>
       <c r="AD10" s="7">
-        <v>5916.4</v>
+        <v>216.6</v>
       </c>
       <c r="AE10" s="4">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="AG10" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="AH10" s="5"/>
+        <v>112</v>
+      </c>
+      <c r="AH10" s="5" t="s">
+        <v>113</v>
+      </c>
       <c r="AI10" s="5"/>
-      <c r="AJ10" s="4"/>
+      <c r="AJ10" s="4">
+        <v>566111704</v>
+      </c>
       <c r="AK10" s="5" t="s">
-        <v>145</v>
+        <v>95</v>
       </c>
       <c r="AL10" s="5" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="AM10" s="6">
-        <v>46077</v>
+        <v>46080</v>
       </c>
       <c r="AN10" s="5" t="s">
         <v>97</v>
@@ -5825,94 +5787,116 @@
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>146</v>
+        <v>310</v>
       </c>
       <c r="C11" s="3">
-        <v>46149</v>
+        <v>46121</v>
       </c>
       <c r="D11" s="4">
-        <v>556897081</v>
+        <v>553095408</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="F11" s="6">
-        <v>46062</v>
+        <v>46069</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>44</v>
+        <v>116</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="K11" s="3">
-        <v>46134</v>
-      </c>
-      <c r="L11" s="12" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="5"/>
+        <v>46246</v>
+      </c>
+      <c r="L11" s="12">
+        <f ca="1">IF($O11="","",$O11-TODAY())</f>
+        <v>134</v>
+      </c>
+      <c r="M11" s="12">
+        <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
+        <v>186</v>
+      </c>
+      <c r="N11" s="12">
+        <f ca="1">IF($C11="","",$C11+120-TODAY())</f>
+        <v>-59</v>
+      </c>
+      <c r="O11" s="6">
+        <v>46434</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="Q11" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="S11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="T11" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="U11" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="V11" s="5" t="s">
         <v>100</v>
       </c>
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
       <c r="Y11" s="5" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="Z11" s="7">
-        <v>5424.4</v>
+        <v>18176.900000000001</v>
       </c>
       <c r="AA11" s="7">
-        <v>0</v>
+        <v>15508.1</v>
       </c>
       <c r="AB11" s="7">
-        <v>0</v>
+        <v>542.44000000000005</v>
       </c>
       <c r="AC11" s="6">
-        <v>46149</v>
+        <v>46121</v>
       </c>
       <c r="AD11" s="7">
-        <v>5424.4</v>
+        <v>2126.36</v>
       </c>
       <c r="AE11" s="4">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="AF11" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="AG11" s="5"/>
+      <c r="AG11" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="AH11" s="5"/>
       <c r="AI11" s="5"/>
-      <c r="AJ11" s="4"/>
+      <c r="AJ11" s="4">
+        <v>557144068</v>
+      </c>
       <c r="AK11" s="5" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="AL11" s="5" t="s">
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="AM11" s="6">
-        <v>46063</v>
+        <v>46099</v>
       </c>
       <c r="AN11" s="5" t="s">
         <v>97</v>
@@ -5920,63 +5904,81 @@
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>152</v>
+        <v>311</v>
       </c>
       <c r="C12" s="3">
-        <v>46112</v>
+        <v>46101</v>
       </c>
       <c r="D12" s="4">
-        <v>553079628</v>
+        <v>550127169</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="F12" s="6">
-        <v>46064</v>
+        <v>46071</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>44</v>
+        <v>122</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="K12" s="3">
-        <v>46244</v>
-      </c>
-      <c r="L12" s="12" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="5"/>
+        <v>46300</v>
+      </c>
+      <c r="L12" s="12">
+        <f ca="1">IF($O12="","",$O12-TODAY())</f>
+        <v>136</v>
+      </c>
+      <c r="M12" s="12">
+        <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
+        <v>166</v>
+      </c>
+      <c r="N12" s="12">
+        <f ca="1">IF($C12="","",$C12+120-TODAY())</f>
+        <v>-79</v>
+      </c>
+      <c r="O12" s="6">
+        <v>46436</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="Q12" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
-      <c r="T12" s="5"/>
-      <c r="U12" s="5"/>
+        <v>90</v>
+      </c>
+      <c r="R12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="S12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="T12" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="U12" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="V12" s="5" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="W12" s="5"/>
       <c r="X12" s="5"/>
       <c r="Y12" s="5" t="s">
-        <v>118</v>
+        <v>51</v>
       </c>
       <c r="Z12" s="7">
-        <v>18176.900000000001</v>
+        <v>6392.96</v>
       </c>
       <c r="AA12" s="7">
         <v>0</v>
@@ -5985,31 +5987,29 @@
         <v>0</v>
       </c>
       <c r="AC12" s="6">
-        <v>46112</v>
+        <v>46101</v>
       </c>
       <c r="AD12" s="7">
-        <v>18176.900000000001</v>
+        <v>6392.96</v>
       </c>
       <c r="AE12" s="4">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="AF12" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG12" s="5" t="s">
-        <v>155</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="AG12" s="5"/>
       <c r="AH12" s="5"/>
       <c r="AI12" s="5"/>
       <c r="AJ12" s="4"/>
       <c r="AK12" s="5" t="s">
-        <v>156</v>
+        <v>125</v>
       </c>
       <c r="AL12" s="5" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="AM12" s="6">
-        <v>46099</v>
+        <v>46093</v>
       </c>
       <c r="AN12" s="5" t="s">
         <v>97</v>
@@ -7152,110 +7152,112 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B2" s="2"/>
+        <v>158</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="C2" s="3">
-        <v>46128</v>
+        <v>46212</v>
       </c>
       <c r="D2" s="4">
-        <v>549835748</v>
+        <v>563274947</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>197</v>
+        <v>133</v>
       </c>
       <c r="F2" s="6">
-        <v>46070</v>
+        <v>46079</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>198</v>
+        <v>43</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>161</v>
+        <v>43</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>198</v>
+        <v>44</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="12">
-        <f t="shared" ref="L2:L11" ca="1" si="0">IF($O2="","",$O2-TODAY())</f>
-        <v>135</v>
+        <f ca="1">IF($O2="","",$O2-TODAY())</f>
+        <v>-131</v>
       </c>
       <c r="M2" s="12">
+        <f ca="1">IF($F2="","",$F2+90-TODAY())</f>
+        <v>-131</v>
+      </c>
+      <c r="N2" s="12">
         <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
-        <v>193</v>
-      </c>
-      <c r="N2" s="12">
-        <f ca="1">IF($C2="","",$C2+120-TODAY())</f>
-        <v>-52</v>
+        <v>277</v>
       </c>
       <c r="O2" s="6">
-        <v>46435</v>
+        <v>46169</v>
       </c>
       <c r="P2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="T2" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>91</v>
       </c>
       <c r="U2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="V2" s="5"/>
+      <c r="V2" s="5" t="s">
+        <v>228</v>
+      </c>
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5" t="s">
         <v>51</v>
       </c>
       <c r="Z2" s="7">
-        <v>2493.33</v>
+        <v>6709.36</v>
       </c>
       <c r="AA2" s="7">
-        <v>2340.02</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="7">
-        <v>153.15</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="6">
-        <v>46128</v>
+        <v>46212</v>
       </c>
       <c r="AD2" s="7">
-        <v>0.16</v>
+        <v>6709.36</v>
       </c>
       <c r="AE2" s="4">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>105</v>
+        <v>213</v>
       </c>
       <c r="AG2" s="5" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="AH2" s="5"/>
       <c r="AI2" s="5"/>
-      <c r="AJ2" s="4">
-        <v>557765015</v>
-      </c>
+      <c r="AJ2" s="4"/>
       <c r="AK2" s="5" t="s">
-        <v>201</v>
+        <v>137</v>
       </c>
       <c r="AL2" s="5" t="s">
-        <v>171</v>
+        <v>230</v>
       </c>
       <c r="AM2" s="6">
-        <v>46072</v>
+        <v>46092</v>
       </c>
       <c r="AN2" s="5" t="s">
         <v>202</v>
@@ -7296,7 +7298,7 @@
         <v>46251</v>
       </c>
       <c r="L3" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O3="","",$O3-TODAY())</f>
         <v>138</v>
       </c>
       <c r="M3" s="12">
@@ -7409,7 +7411,7 @@
         <v>46195</v>
       </c>
       <c r="L4" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O4="","",$O4-TODAY())</f>
         <v>144</v>
       </c>
       <c r="M4" s="12">
@@ -7530,7 +7532,7 @@
         <v>46247</v>
       </c>
       <c r="L5" s="12">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF($O5="","",$O5-TODAY())</f>
         <v>-151</v>
       </c>
       <c r="M5" s="12">
@@ -7608,61 +7610,61 @@
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C6" s="3">
-        <v>46233</v>
+        <v>46189</v>
       </c>
       <c r="D6" s="4">
-        <v>551412333</v>
+        <v>562083380</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="F6" s="6">
-        <v>46072</v>
+        <v>46080</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>141</v>
+        <v>68</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>141</v>
+        <v>68</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="K6" s="3">
-        <v>46192</v>
+        <v>46247</v>
       </c>
       <c r="L6" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-138</v>
+        <f ca="1">IF($O6="","",$O6-TODAY())</f>
+        <v>-130</v>
       </c>
       <c r="M6" s="12">
-        <f ca="1">IF($C6="","",$C6+180-TODAY())</f>
-        <v>113</v>
+        <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
+        <v>254</v>
       </c>
       <c r="N6" s="12">
         <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>298</v>
+        <v>254</v>
       </c>
       <c r="O6" s="6">
-        <v>46162</v>
+        <v>46170</v>
       </c>
       <c r="P6" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>142</v>
+        <v>70</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>143</v>
+        <v>49</v>
       </c>
       <c r="S6" s="5" t="s">
         <v>50</v>
@@ -7674,7 +7676,7 @@
         <v>50</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="W6" s="5"/>
       <c r="X6" s="5"/>
@@ -7682,7 +7684,7 @@
         <v>51</v>
       </c>
       <c r="Z6" s="7">
-        <v>6297.27</v>
+        <v>7623.07</v>
       </c>
       <c r="AA6" s="7">
         <v>0</v>
@@ -7691,35 +7693,29 @@
         <v>0</v>
       </c>
       <c r="AC6" s="6">
-        <v>46142</v>
+        <v>46189</v>
       </c>
       <c r="AD6" s="7">
-        <v>6297.27</v>
+        <v>7623.07</v>
       </c>
       <c r="AE6" s="4">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="AF6" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="AG6" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="AH6" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="AI6" s="5" t="s">
-        <v>136</v>
-      </c>
+      <c r="AG6" s="5"/>
+      <c r="AH6" s="5"/>
+      <c r="AI6" s="5"/>
       <c r="AJ6" s="4"/>
       <c r="AK6" s="5" t="s">
-        <v>215</v>
+        <v>53</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="AM6" s="6">
-        <v>46084</v>
+        <v>46083</v>
       </c>
       <c r="AN6" s="5" t="s">
         <v>202</v>
@@ -7727,59 +7723,61 @@
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>158</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>226</v>
+        <v>306</v>
       </c>
       <c r="C7" s="3">
-        <v>46212</v>
+        <v>46218</v>
       </c>
       <c r="D7" s="4">
-        <v>563274947</v>
+        <v>564578362</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>133</v>
+        <v>235</v>
       </c>
       <c r="F7" s="6">
-        <v>46079</v>
+        <v>46057</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>43</v>
+        <v>236</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>43</v>
+        <v>236</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="K7" s="3"/>
+        <v>237</v>
+      </c>
+      <c r="K7" s="3">
+        <v>46285</v>
+      </c>
       <c r="L7" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-131</v>
+        <f ca="1">IF($O7="","",$O7-TODAY())</f>
+        <v>-123</v>
       </c>
       <c r="M7" s="12">
-        <f ca="1">IF($F7="","",$F7+90-TODAY())</f>
-        <v>-131</v>
+        <f ca="1">IF($F7="","",$F7+365-TODAY())</f>
+        <v>122</v>
       </c>
       <c r="N7" s="12">
-        <f ca="1">IF($C7="","",$C7+365-TODAY())</f>
-        <v>277</v>
+        <f ca="1">IF($F7="","",$F7+365-TODAY())</f>
+        <v>122</v>
       </c>
       <c r="O7" s="6">
-        <v>46169</v>
+        <v>46177</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>47</v>
+        <v>238</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="S7" s="5" t="s">
         <v>48</v>
@@ -7788,18 +7786,16 @@
         <v>49</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="V7" s="5" t="s">
-        <v>228</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="V7" s="5"/>
       <c r="W7" s="5"/>
       <c r="X7" s="5"/>
       <c r="Y7" s="5" t="s">
         <v>51</v>
       </c>
       <c r="Z7" s="7">
-        <v>6709.36</v>
+        <v>1433.32</v>
       </c>
       <c r="AA7" s="7">
         <v>0</v>
@@ -7808,31 +7804,31 @@
         <v>0</v>
       </c>
       <c r="AC7" s="6">
-        <v>46212</v>
+        <v>46218</v>
       </c>
       <c r="AD7" s="7">
-        <v>6709.36</v>
+        <v>1433.32</v>
       </c>
       <c r="AE7" s="4">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="AF7" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AG7" s="5" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="AH7" s="5"/>
       <c r="AI7" s="5"/>
       <c r="AJ7" s="4"/>
       <c r="AK7" s="5" t="s">
-        <v>137</v>
+        <v>240</v>
       </c>
       <c r="AL7" s="5" t="s">
-        <v>230</v>
+        <v>171</v>
       </c>
       <c r="AM7" s="6">
-        <v>46092</v>
+        <v>46077</v>
       </c>
       <c r="AN7" s="5" t="s">
         <v>202</v>
@@ -7843,78 +7839,65 @@
         <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="C8" s="3">
-        <v>46189</v>
+        <v>46107</v>
       </c>
       <c r="D8" s="4">
-        <v>562083380</v>
+        <v>552275426</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="F8" s="6">
-        <v>46080</v>
+        <v>46079</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>68</v>
+        <v>249</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>68</v>
+        <v>249</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>233</v>
+        <v>250</v>
       </c>
       <c r="K8" s="3">
-        <v>46247</v>
-      </c>
-      <c r="L8" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-130</v>
-      </c>
-      <c r="M8" s="12">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
-        <v>254</v>
-      </c>
+        <v>46195</v>
+      </c>
+      <c r="L8" s="12" t="str">
+        <f ca="1">IF($O8="","",$O8-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M8" s="12"/>
       <c r="N8" s="12">
-        <f ca="1">IF($C8="","",$C8+365-TODAY())</f>
-        <v>254</v>
-      </c>
-      <c r="O8" s="6">
-        <v>46170</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>46</v>
-      </c>
+        <f ca="1">IF($C8="","",$C8+180-TODAY())</f>
+        <v>-13</v>
+      </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="5"/>
       <c r="Q8" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>50</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
       <c r="T8" s="5" t="s">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="U8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="V8" s="5" t="s">
-        <v>234</v>
-      </c>
+      <c r="V8" s="5"/>
       <c r="W8" s="5"/>
       <c r="X8" s="5"/>
       <c r="Y8" s="5" t="s">
         <v>51</v>
       </c>
       <c r="Z8" s="7">
-        <v>7623.07</v>
+        <v>1758.12</v>
       </c>
       <c r="AA8" s="7">
         <v>0</v>
@@ -7923,29 +7906,31 @@
         <v>0</v>
       </c>
       <c r="AC8" s="6">
-        <v>46189</v>
+        <v>46107</v>
       </c>
       <c r="AD8" s="7">
-        <v>7623.07</v>
+        <v>1758.12</v>
       </c>
       <c r="AE8" s="4">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AF8" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="AG8" s="5"/>
+        <v>213</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>252</v>
+      </c>
       <c r="AH8" s="5"/>
       <c r="AI8" s="5"/>
       <c r="AJ8" s="4"/>
       <c r="AK8" s="5" t="s">
-        <v>53</v>
+        <v>137</v>
       </c>
       <c r="AL8" s="5" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
       <c r="AM8" s="6">
-        <v>46083</v>
+        <v>46092</v>
       </c>
       <c r="AN8" s="5" t="s">
         <v>202</v>
@@ -7953,70 +7938,66 @@
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>306</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="B9" s="2"/>
       <c r="C9" s="3">
-        <v>46218</v>
+        <v>46128</v>
       </c>
       <c r="D9" s="4">
-        <v>564578362</v>
+        <v>549835748</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>235</v>
+        <v>197</v>
       </c>
       <c r="F9" s="6">
-        <v>46057</v>
+        <v>46070</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>236</v>
+        <v>198</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>236</v>
+        <v>161</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>44</v>
+        <v>198</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="K9" s="3">
-        <v>46285</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="K9" s="3"/>
       <c r="L9" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-123</v>
+        <f ca="1">IF($O9="","",$O9-TODAY())</f>
+        <v>135</v>
       </c>
       <c r="M9" s="12">
-        <f ca="1">IF($F9="","",$F9+365-TODAY())</f>
-        <v>122</v>
+        <f ca="1">IF($C9="","",$C9+365-TODAY())</f>
+        <v>193</v>
       </c>
       <c r="N9" s="12">
-        <f ca="1">IF($F9="","",$F9+365-TODAY())</f>
-        <v>122</v>
+        <f ca="1">IF($C9="","",$C9+120-TODAY())</f>
+        <v>-52</v>
       </c>
       <c r="O9" s="6">
-        <v>46177</v>
+        <v>46435</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>238</v>
+        <v>90</v>
       </c>
       <c r="R9" s="5" t="s">
         <v>49</v>
       </c>
       <c r="S9" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>49</v>
+        <v>91</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
@@ -8025,40 +8006,42 @@
         <v>51</v>
       </c>
       <c r="Z9" s="7">
-        <v>1433.32</v>
+        <v>2493.33</v>
       </c>
       <c r="AA9" s="7">
-        <v>0</v>
+        <v>2340.02</v>
       </c>
       <c r="AB9" s="7">
-        <v>0</v>
+        <v>153.15</v>
       </c>
       <c r="AC9" s="6">
-        <v>46218</v>
+        <v>46128</v>
       </c>
       <c r="AD9" s="7">
-        <v>1433.32</v>
+        <v>0.16</v>
       </c>
       <c r="AE9" s="4">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="AF9" s="5" t="s">
-        <v>212</v>
+        <v>105</v>
       </c>
       <c r="AG9" s="5" t="s">
-        <v>239</v>
+        <v>200</v>
       </c>
       <c r="AH9" s="5"/>
       <c r="AI9" s="5"/>
-      <c r="AJ9" s="4"/>
+      <c r="AJ9" s="4">
+        <v>557765015</v>
+      </c>
       <c r="AK9" s="5" t="s">
-        <v>240</v>
+        <v>201</v>
       </c>
       <c r="AL9" s="5" t="s">
         <v>171</v>
       </c>
       <c r="AM9" s="6">
-        <v>46077</v>
+        <v>46072</v>
       </c>
       <c r="AN9" s="5" t="s">
         <v>202</v>
@@ -8069,58 +8052,58 @@
         <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>241</v>
+        <v>222</v>
       </c>
       <c r="C10" s="3">
-        <v>46142</v>
+        <v>46233</v>
       </c>
       <c r="D10" s="4">
-        <v>551321878</v>
+        <v>551412333</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>242</v>
+        <v>223</v>
       </c>
       <c r="F10" s="6">
-        <v>46058</v>
+        <v>46072</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>243</v>
+        <v>141</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>243</v>
+        <v>141</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="K10" s="3">
-        <v>46195</v>
+        <v>46192</v>
       </c>
       <c r="L10" s="12">
-        <f t="shared" ca="1" si="0"/>
-        <v>-152</v>
+        <f ca="1">IF($O10="","",$O10-TODAY())</f>
+        <v>-138</v>
       </c>
       <c r="M10" s="12">
-        <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>207</v>
+        <f ca="1">IF($C10="","",$C10+180-TODAY())</f>
+        <v>113</v>
       </c>
       <c r="N10" s="12">
         <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>207</v>
+        <v>298</v>
       </c>
       <c r="O10" s="6">
-        <v>46148</v>
+        <v>46162</v>
       </c>
       <c r="P10" s="5" t="s">
         <v>46</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>245</v>
+        <v>142</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="S10" s="5" t="s">
         <v>50</v>
@@ -8131,14 +8114,16 @@
       <c r="U10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="V10" s="5"/>
+      <c r="V10" s="5" t="s">
+        <v>225</v>
+      </c>
       <c r="W10" s="5"/>
       <c r="X10" s="5"/>
       <c r="Y10" s="5" t="s">
         <v>51</v>
       </c>
       <c r="Z10" s="7">
-        <v>12527.55</v>
+        <v>6297.27</v>
       </c>
       <c r="AA10" s="7">
         <v>0</v>
@@ -8150,10 +8135,10 @@
         <v>46142</v>
       </c>
       <c r="AD10" s="7">
-        <v>12527.55</v>
+        <v>6297.27</v>
       </c>
       <c r="AE10" s="4">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="AF10" s="5" t="s">
         <v>212</v>
@@ -8162,10 +8147,10 @@
         <v>213</v>
       </c>
       <c r="AH10" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="AI10" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="AI10" s="5" t="s">
-        <v>246</v>
       </c>
       <c r="AJ10" s="4"/>
       <c r="AK10" s="5" t="s">
@@ -8175,7 +8160,7 @@
         <v>171</v>
       </c>
       <c r="AM10" s="6">
-        <v>46083</v>
+        <v>46084</v>
       </c>
       <c r="AN10" s="5" t="s">
         <v>202</v>
@@ -8183,56 +8168,67 @@
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C11" s="3">
-        <v>46107</v>
+        <v>46142</v>
       </c>
       <c r="D11" s="4">
-        <v>552275426</v>
+        <v>551321878</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="F11" s="6">
-        <v>46079</v>
+        <v>46058</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>44</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="K11" s="3">
         <v>46195</v>
       </c>
-      <c r="L11" s="12" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="M11" s="12"/>
+      <c r="L11" s="12">
+        <f ca="1">IF($O11="","",$O11-TODAY())</f>
+        <v>-152</v>
+      </c>
+      <c r="M11" s="12">
+        <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
+        <v>207</v>
+      </c>
       <c r="N11" s="12">
-        <f ca="1">IF($C11="","",$C11+180-TODAY())</f>
-        <v>-13</v>
-      </c>
-      <c r="O11" s="6"/>
-      <c r="P11" s="5"/>
+        <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
+        <v>207</v>
+      </c>
+      <c r="O11" s="6">
+        <v>46148</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="Q11" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
+        <v>245</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="S11" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="T11" s="5" t="s">
-        <v>143</v>
+        <v>49</v>
       </c>
       <c r="U11" s="5" t="s">
         <v>50</v>
@@ -8244,7 +8240,7 @@
         <v>51</v>
       </c>
       <c r="Z11" s="7">
-        <v>1758.12</v>
+        <v>12527.55</v>
       </c>
       <c r="AA11" s="7">
         <v>0</v>
@@ -8253,31 +8249,35 @@
         <v>0</v>
       </c>
       <c r="AC11" s="6">
-        <v>46107</v>
+        <v>46142</v>
       </c>
       <c r="AD11" s="7">
-        <v>1758.12</v>
+        <v>12527.55</v>
       </c>
       <c r="AE11" s="4">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="AF11" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AG11" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="AG11" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="AH11" s="5"/>
-      <c r="AI11" s="5"/>
+      <c r="AH11" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="AI11" s="5" t="s">
+        <v>246</v>
+      </c>
       <c r="AJ11" s="4"/>
       <c r="AK11" s="5" t="s">
-        <v>137</v>
+        <v>215</v>
       </c>
       <c r="AL11" s="5" t="s">
-        <v>230</v>
+        <v>171</v>
       </c>
       <c r="AM11" s="6">
-        <v>46092</v>
+        <v>46083</v>
       </c>
       <c r="AN11" s="5" t="s">
         <v>202</v>
@@ -8555,41 +8555,41 @@
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>203</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
       <c r="C2" s="3">
         <v>46211</v>
       </c>
       <c r="D2" s="4">
-        <v>563152890</v>
+        <v>563161793</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
       <c r="F2" s="6">
-        <v>46057</v>
+        <v>46065</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>43</v>
+        <v>272</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>161</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>43</v>
+        <v>272</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>255</v>
       </c>
       <c r="K2" s="3">
-        <v>46196</v>
+        <v>46251</v>
       </c>
       <c r="L2" s="12">
         <f ca="1">IF($O2="","",$O2-TODAY())</f>
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="M2" s="12">
         <f ca="1">IF($C2="","",$C2+365-TODAY())</f>
@@ -8600,7 +8600,7 @@
         <v>31</v>
       </c>
       <c r="O2" s="6">
-        <v>46422</v>
+        <v>46430</v>
       </c>
       <c r="P2" s="5" t="s">
         <v>49</v>
@@ -8630,10 +8630,10 @@
         <v>1294.23</v>
       </c>
       <c r="AA2" s="7">
-        <v>1127.69</v>
+        <v>1131</v>
       </c>
       <c r="AB2" s="7">
-        <v>130.80000000000001</v>
+        <v>127.49</v>
       </c>
       <c r="AC2" s="6">
         <v>46211</v>
@@ -8642,31 +8642,31 @@
         <v>35.74</v>
       </c>
       <c r="AE2" s="4">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="AF2" s="5" t="s">
         <v>256</v>
       </c>
       <c r="AG2" s="5" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="AH2" s="5" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="AI2" s="5" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
       <c r="AJ2" s="4">
-        <v>566075115</v>
+        <v>566075130</v>
       </c>
       <c r="AK2" s="5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="AL2" s="5" t="s">
-        <v>157</v>
+        <v>65</v>
       </c>
       <c r="AM2" s="6">
-        <v>46072</v>
+        <v>46076</v>
       </c>
       <c r="AN2" s="5" t="s">
         <v>261</v>
@@ -8683,32 +8683,32 @@
         <v>46211</v>
       </c>
       <c r="D3" s="4">
-        <v>563153622</v>
+        <v>563152890</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="F3" s="6">
-        <v>46065</v>
+        <v>46057</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>161</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="K3" s="3">
         <v>46196</v>
       </c>
       <c r="L3" s="12">
         <f ca="1">IF($O3="","",$O3-TODAY())</f>
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="M3" s="12">
         <f ca="1">IF($C3="","",$C3+365-TODAY())</f>
@@ -8719,7 +8719,7 @@
         <v>31</v>
       </c>
       <c r="O3" s="6">
-        <v>46430</v>
+        <v>46422</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>49</v>
@@ -8746,40 +8746,46 @@
         <v>51</v>
       </c>
       <c r="Z3" s="7">
-        <v>2943.43</v>
+        <v>1294.23</v>
       </c>
       <c r="AA3" s="7">
-        <v>2603.25</v>
+        <v>1127.69</v>
       </c>
       <c r="AB3" s="7">
-        <v>265.7</v>
+        <v>130.80000000000001</v>
       </c>
       <c r="AC3" s="6">
         <v>46211</v>
       </c>
       <c r="AD3" s="7">
-        <v>74.48</v>
+        <v>35.74</v>
       </c>
       <c r="AE3" s="4">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="AF3" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="AG3" s="5"/>
-      <c r="AH3" s="5"/>
-      <c r="AI3" s="5"/>
+        <v>256</v>
+      </c>
+      <c r="AG3" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="AH3" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>259</v>
+      </c>
       <c r="AJ3" s="4">
-        <v>565916751</v>
+        <v>566075115</v>
       </c>
       <c r="AK3" s="5" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AL3" s="5" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="AM3" s="6">
-        <v>46119</v>
+        <v>46072</v>
       </c>
       <c r="AN3" s="5" t="s">
         <v>261</v>
@@ -8793,16 +8799,16 @@
         <v>253</v>
       </c>
       <c r="C4" s="3">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="D4" s="4">
-        <v>563152081</v>
+        <v>563153622</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="F4" s="6">
-        <v>46070</v>
+        <v>46065</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>107</v>
@@ -8814,25 +8820,25 @@
         <v>107</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="K4" s="3">
         <v>46196</v>
       </c>
       <c r="L4" s="12">
         <f ca="1">IF($O4="","",$O4-TODAY())</f>
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="M4" s="12">
         <f ca="1">IF($C4="","",$C4+365-TODAY())</f>
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="N4" s="12">
         <f ca="1">IF($C4="","",$C4+120-TODAY())</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O4" s="6">
-        <v>46435</v>
+        <v>46430</v>
       </c>
       <c r="P4" s="5" t="s">
         <v>49</v>
@@ -8859,40 +8865,40 @@
         <v>51</v>
       </c>
       <c r="Z4" s="7">
-        <v>1294.23</v>
+        <v>2943.43</v>
       </c>
       <c r="AA4" s="7">
-        <v>1131</v>
+        <v>2603.25</v>
       </c>
       <c r="AB4" s="7">
-        <v>127.49</v>
+        <v>265.7</v>
       </c>
       <c r="AC4" s="6">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="AD4" s="7">
-        <v>35.74</v>
+        <v>74.48</v>
       </c>
       <c r="AE4" s="4">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AG4" s="5"/>
       <c r="AH4" s="5"/>
       <c r="AI4" s="5"/>
       <c r="AJ4" s="4">
-        <v>566075094</v>
+        <v>565916751</v>
       </c>
       <c r="AK4" s="5" t="s">
-        <v>53</v>
+        <v>265</v>
       </c>
       <c r="AL4" s="5" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="AM4" s="6">
-        <v>46076</v>
+        <v>46119</v>
       </c>
       <c r="AN4" s="5" t="s">
         <v>261</v>
@@ -8909,32 +8915,32 @@
         <v>46210</v>
       </c>
       <c r="D5" s="4">
-        <v>563152473</v>
+        <v>563152081</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F5" s="6">
-        <v>46071</v>
+        <v>46070</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>161</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="K5" s="3">
         <v>46196</v>
       </c>
       <c r="L5" s="12">
         <f ca="1">IF($O5="","",$O5-TODAY())</f>
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M5" s="12">
         <f ca="1">IF($C5="","",$C5+365-TODAY())</f>
@@ -8945,7 +8951,7 @@
         <v>30</v>
       </c>
       <c r="O5" s="6">
-        <v>46436</v>
+        <v>46435</v>
       </c>
       <c r="P5" s="5" t="s">
         <v>49</v>
@@ -8972,40 +8978,40 @@
         <v>51</v>
       </c>
       <c r="Z5" s="7">
-        <v>879.06</v>
+        <v>1294.23</v>
       </c>
       <c r="AA5" s="7">
-        <v>758.3</v>
+        <v>1131</v>
       </c>
       <c r="AB5" s="7">
-        <v>94.84</v>
+        <v>127.49</v>
       </c>
       <c r="AC5" s="6">
         <v>46210</v>
       </c>
       <c r="AD5" s="7">
-        <v>25.92</v>
+        <v>35.74</v>
       </c>
       <c r="AE5" s="4">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AF5" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="AG5" s="5"/>
       <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
       <c r="AJ5" s="4">
-        <v>566075128</v>
+        <v>566075094</v>
       </c>
       <c r="AK5" s="5" t="s">
-        <v>260</v>
+        <v>53</v>
       </c>
       <c r="AL5" s="5" t="s">
-        <v>157</v>
+        <v>72</v>
       </c>
       <c r="AM5" s="6">
-        <v>46119</v>
+        <v>46076</v>
       </c>
       <c r="AN5" s="5" t="s">
         <v>261</v>
@@ -9013,52 +9019,52 @@
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>203</v>
+        <v>114</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="C6" s="3">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="D6" s="4">
-        <v>563161793</v>
+        <v>563152473</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="F6" s="6">
-        <v>46065</v>
+        <v>46071</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>272</v>
+        <v>43</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>161</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>272</v>
+        <v>43</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K6" s="3">
-        <v>46251</v>
+        <v>46196</v>
       </c>
       <c r="L6" s="12">
         <f ca="1">IF($O6="","",$O6-TODAY())</f>
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="M6" s="12">
         <f ca="1">IF($C6="","",$C6+365-TODAY())</f>
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="N6" s="12">
         <f ca="1">IF($C6="","",$C6+120-TODAY())</f>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O6" s="6">
-        <v>46430</v>
+        <v>46436</v>
       </c>
       <c r="P6" s="5" t="s">
         <v>49</v>
@@ -9085,46 +9091,40 @@
         <v>51</v>
       </c>
       <c r="Z6" s="7">
-        <v>1294.23</v>
+        <v>879.06</v>
       </c>
       <c r="AA6" s="7">
-        <v>1131</v>
+        <v>758.3</v>
       </c>
       <c r="AB6" s="7">
-        <v>127.49</v>
+        <v>94.84</v>
       </c>
       <c r="AC6" s="6">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="AD6" s="7">
-        <v>35.74</v>
+        <v>25.92</v>
       </c>
       <c r="AE6" s="4">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="AG6" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="AH6" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="AI6" s="5" t="s">
-        <v>275</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="AG6" s="5"/>
+      <c r="AH6" s="5"/>
+      <c r="AI6" s="5"/>
       <c r="AJ6" s="4">
-        <v>566075130</v>
+        <v>566075128</v>
       </c>
       <c r="AK6" s="5" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="AM6" s="6">
-        <v>46076</v>
+        <v>46119</v>
       </c>
       <c r="AN6" s="5" t="s">
         <v>261</v>
@@ -9268,7 +9268,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>279</v>
       </c>
@@ -9311,7 +9311,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>287</v>
       </c>

</xml_diff>

<commit_message>
Delete Finalized claims with a Latest Date Worked and a note of just PAID
Removes the 5 matching claims (551104780, 557717115, 556761529,
562882369, 563836350) from their monthly sheets (Feb DME, Mar DME,
Jun BH, Jun ORTHO) and from the master. Rows below move up with their
formulas; filter, validation and deadline-colour ranges shrink to fit.
Read Me claim totals and deadline-band counts updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgCgUMEP34hb7McfZTNVaf
</commit_message>
<xml_diff>
--- a/SPC26S1 - 02 February.xlsx
+++ b/SPC26S1 - 02 February.xlsx
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BH!$A$1:$AO$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DME!$A$1:$AO$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DME!$A$1:$AO$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">GAE!$A$1:$AO$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">ORTHO!$A$1:$AO$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">US!$A$1:$AO$6</definedName>
@@ -1841,7 +1841,7 @@
     <t>2026-02 February - Specialty Claims</t>
   </si>
   <si>
-    <t>39 claims with a date of service in 2026-02 February, split into one sheet per specialty: BH, DME, GAE, ORTHO, US.</t>
+    <t>38 claims with a date of service in 2026-02 February, split into one sheet per specialty: BH, DME, GAE, ORTHO, US.</t>
   </si>
   <si>
     <t>Row order - work queue, then timely filing deadline</t>
@@ -1859,7 +1859,7 @@
     <t xml:space="preserve">    2 - Due in 6-30 days: 0</t>
   </si>
   <si>
-    <t xml:space="preserve">    3 - Due in 31+ days: 19</t>
+    <t xml:space="preserve">    3 - Due in 31+ days: 18</t>
   </si>
   <si>
     <t xml:space="preserve">    4 - Past deadline: 17</t>
@@ -1916,7 +1916,7 @@
     <t>How this file feeds the master</t>
   </si>
   <si>
-    <t>'ALL Claims 2026-S1 - Master.xlsx' (same folder) holds all 482 claims for 2026 S1. Its Claim Status and Notes columns are formulas that read this file, so anything you type in columns A and B here shows up there. Keep both files in the same folder, keep the file name unchanged, and save this file before opening the master.</t>
+    <t>'ALL Claims 2026-S1 - Master.xlsx' (same folder) holds all 477 claims for 2026 S1. Its Claim Status and Notes columns are formulas that read this file, so anything you type in columns A and B here shows up there. Keep both files in the same folder, keep the file name unchanged, and save this file before opening the master.</t>
   </si>
   <si>
     <t>The link is matched on Primary Claim ID, not on row position, so sorting and filtering these sheets is safe. Do not edit that column, and do not rename the specialty sheet tabs.</t>
@@ -4622,7 +4622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AN12"/>
+  <dimension ref="A1:AN11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5669,34 +5669,34 @@
         <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>114</v>
+        <v>310</v>
       </c>
       <c r="C10" s="3">
-        <v>46133</v>
+        <v>46121</v>
       </c>
       <c r="D10" s="4">
-        <v>551104780</v>
+        <v>553095408</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F10" s="6">
         <v>46069</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>88</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="K10" s="3">
-        <v>46261</v>
+        <v>46246</v>
       </c>
       <c r="L10" s="12">
         <f ca="1">IF($O10="","",$O10-TODAY())</f>
@@ -5704,11 +5704,11 @@
       </c>
       <c r="M10" s="12">
         <f ca="1">IF($C10="","",$C10+365-TODAY())</f>
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="N10" s="12">
         <f ca="1">IF($C10="","",$C10+120-TODAY())</f>
-        <v>-47</v>
+        <v>-59</v>
       </c>
       <c r="O10" s="6">
         <v>46434</v>
@@ -5732,54 +5732,50 @@
         <v>50</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="W10" s="5" t="s">
-        <v>110</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="W10" s="5"/>
       <c r="X10" s="5"/>
       <c r="Y10" s="5" t="s">
-        <v>51</v>
+        <v>118</v>
       </c>
       <c r="Z10" s="7">
-        <v>1082.98</v>
+        <v>18176.900000000001</v>
       </c>
       <c r="AA10" s="7">
-        <v>17.32</v>
+        <v>15508.1</v>
       </c>
       <c r="AB10" s="7">
-        <v>849.06</v>
+        <v>542.44000000000005</v>
       </c>
       <c r="AC10" s="6">
-        <v>46133</v>
+        <v>46121</v>
       </c>
       <c r="AD10" s="7">
-        <v>216.6</v>
+        <v>2126.36</v>
       </c>
       <c r="AE10" s="4">
         <v>173</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="AG10" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="AH10" s="5" t="s">
-        <v>113</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="AH10" s="5"/>
       <c r="AI10" s="5"/>
       <c r="AJ10" s="4">
-        <v>566111704</v>
+        <v>557144068</v>
       </c>
       <c r="AK10" s="5" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="AL10" s="5" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="AM10" s="6">
-        <v>46080</v>
+        <v>46099</v>
       </c>
       <c r="AN10" s="5" t="s">
         <v>97</v>
@@ -5790,49 +5786,49 @@
         <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C11" s="3">
-        <v>46121</v>
+        <v>46101</v>
       </c>
       <c r="D11" s="4">
-        <v>553095408</v>
+        <v>550127169</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F11" s="6">
-        <v>46069</v>
+        <v>46071</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>88</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="K11" s="3">
-        <v>46246</v>
+        <v>46300</v>
       </c>
       <c r="L11" s="12">
         <f ca="1">IF($O11="","",$O11-TODAY())</f>
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="M11" s="12">
         <f ca="1">IF($C11="","",$C11+365-TODAY())</f>
-        <v>186</v>
+        <v>166</v>
       </c>
       <c r="N11" s="12">
         <f ca="1">IF($C11="","",$C11+120-TODAY())</f>
-        <v>-59</v>
+        <v>-79</v>
       </c>
       <c r="O11" s="6">
-        <v>46434</v>
+        <v>46436</v>
       </c>
       <c r="P11" s="5" t="s">
         <v>49</v>
@@ -5853,171 +5849,54 @@
         <v>50</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
       <c r="Y11" s="5" t="s">
-        <v>118</v>
+        <v>51</v>
       </c>
       <c r="Z11" s="7">
-        <v>18176.900000000001</v>
+        <v>6392.96</v>
       </c>
       <c r="AA11" s="7">
-        <v>15508.1</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="7">
-        <v>542.44000000000005</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="6">
-        <v>46121</v>
+        <v>46101</v>
       </c>
       <c r="AD11" s="7">
-        <v>2126.36</v>
+        <v>6392.96</v>
       </c>
       <c r="AE11" s="4">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="AF11" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG11" s="5" t="s">
-        <v>105</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="AG11" s="5"/>
       <c r="AH11" s="5"/>
       <c r="AI11" s="5"/>
-      <c r="AJ11" s="4">
-        <v>557144068</v>
-      </c>
+      <c r="AJ11" s="4"/>
       <c r="AK11" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="AL11" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="AM11" s="6">
-        <v>46099</v>
+        <v>46093</v>
       </c>
       <c r="AN11" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C12" s="3">
-        <v>46101</v>
-      </c>
-      <c r="D12" s="4">
-        <v>550127169</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F12" s="6">
-        <v>46071</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="K12" s="3">
-        <v>46300</v>
-      </c>
-      <c r="L12" s="12">
-        <f ca="1">IF($O12="","",$O12-TODAY())</f>
-        <v>136</v>
-      </c>
-      <c r="M12" s="12">
-        <f ca="1">IF($C12="","",$C12+365-TODAY())</f>
-        <v>166</v>
-      </c>
-      <c r="N12" s="12">
-        <f ca="1">IF($C12="","",$C12+120-TODAY())</f>
-        <v>-79</v>
-      </c>
-      <c r="O12" s="6">
-        <v>46436</v>
-      </c>
-      <c r="P12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q12" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="R12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="T12" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="U12" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="V12" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="W12" s="5"/>
-      <c r="X12" s="5"/>
-      <c r="Y12" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z12" s="7">
-        <v>6392.96</v>
-      </c>
-      <c r="AA12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="6">
-        <v>46101</v>
-      </c>
-      <c r="AD12" s="7">
-        <v>6392.96</v>
-      </c>
-      <c r="AE12" s="4">
-        <v>171</v>
-      </c>
-      <c r="AF12" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="AG12" s="5"/>
-      <c r="AH12" s="5"/>
-      <c r="AI12" s="5"/>
-      <c r="AJ12" s="4"/>
-      <c r="AK12" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="AL12" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="AM12" s="6">
-        <v>46093</v>
-      </c>
-      <c r="AN12" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AN12" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="L2:L12">
+  <autoFilter ref="A1:AN11" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="L2:L11">
     <cfRule type="expression" dxfId="79" priority="1">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
@@ -6034,7 +5913,7 @@
       <formula>$L2=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M12">
+  <conditionalFormatting sqref="M2:M11">
     <cfRule type="expression" dxfId="74" priority="6">
       <formula>AND($M2&lt;&gt;"", $M2&gt;=0, $M2&lt;=5)</formula>
     </cfRule>
@@ -6051,7 +5930,7 @@
       <formula>$M2=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N12">
+  <conditionalFormatting sqref="N2:N11">
     <cfRule type="expression" dxfId="69" priority="11">
       <formula>AND($N2&lt;&gt;"", $N2&gt;=0, $N2&lt;=5)</formula>
     </cfRule>
@@ -6068,7 +5947,7 @@
       <formula>$N2=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:U12">
+  <conditionalFormatting sqref="O2:U11">
     <cfRule type="expression" dxfId="64" priority="16">
       <formula>AND($L2&lt;&gt;"", $L2&gt;=0, $L2&lt;=5)</formula>
     </cfRule>
@@ -6112,7 +5991,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Claim Status" prompt="Pick a status, or type a new one." sqref="A2:A12" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Claim Status" prompt="Pick a status, or type a new one." sqref="A2:A11" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Denied,Finalized,PAID,Pending,Received,Rejected,Under Review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>